<commit_message>
Add configurable tenant logo
</commit_message>
<xml_diff>
--- a/tenants/sjc/reports/OSO/templates/v1.xlsx
+++ b/tenants/sjc/reports/OSO/templates/v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaiqu\OneDrive\Área de Trabalho\Stravia Consultoria\01. Projetos\01.14 Goal Bus - API\Github\excel-report-api\tenants\sjc\reports\OSO\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF50ED0-F3B7-4510-B349-6EE4C6E27FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CEAE44-B77D-4585-9C76-3AE93CAA3DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-3570" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -147,7 +147,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -176,12 +176,6 @@
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -366,50 +360,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="20" fontId="7" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="6" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="20" fontId="7" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -428,37 +404,37 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="20" fontId="9" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="8" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="9" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="8" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="8" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="9" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="8" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -485,18 +461,18 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>775221</xdr:colOff>
+      <xdr:colOff>477565</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>10583</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>860946</xdr:colOff>
+      <xdr:colOff>563290</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>210170</xdr:rowOff>
+      <xdr:rowOff>199587</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -525,8 +501,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17205846" y="10583"/>
-          <a:ext cx="3743325" cy="694887"/>
+          <a:off x="16908190" y="0"/>
+          <a:ext cx="3752850" cy="699650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -739,348 +715,206 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AO15"/>
+  <dimension ref="A1:X15"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" style="5" customWidth="1"/>
-    <col min="3" max="8" width="12.7109375" style="5" customWidth="1"/>
-    <col min="9" max="9" width="30.7109375" style="5" customWidth="1"/>
-    <col min="10" max="21" width="13.7109375" style="5" customWidth="1"/>
-    <col min="22" max="22" width="20" style="5" customWidth="1"/>
-    <col min="23" max="41" width="9.140625" style="5" customWidth="1"/>
-    <col min="42" max="16384" width="12.5703125" style="5"/>
+    <col min="1" max="1" width="12.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="30.7109375" style="3" customWidth="1"/>
+    <col min="3" max="8" width="12.7109375" style="3" customWidth="1"/>
+    <col min="9" max="9" width="30.7109375" style="3" customWidth="1"/>
+    <col min="10" max="21" width="13.7109375" style="3" customWidth="1"/>
+    <col min="22" max="16384" width="12.5703125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18"/>
-      <c r="T1" s="18"/>
-      <c r="U1" s="18"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="4"/>
-      <c r="Y1" s="4"/>
-      <c r="Z1" s="4"/>
-      <c r="AA1" s="4"/>
-      <c r="AB1" s="4"/>
-      <c r="AC1" s="4"/>
-      <c r="AD1" s="4"/>
-      <c r="AE1" s="4"/>
-      <c r="AF1" s="4"/>
-      <c r="AG1" s="4"/>
-      <c r="AH1" s="4"/>
-      <c r="AI1" s="4"/>
-      <c r="AJ1" s="4"/>
-      <c r="AK1" s="4"/>
-      <c r="AL1" s="4"/>
-      <c r="AM1" s="4"/>
-      <c r="AN1" s="4"/>
-      <c r="AO1" s="4"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
     </row>
-    <row r="2" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="18"/>
-      <c r="S2" s="18"/>
-      <c r="T2" s="18"/>
-      <c r="U2" s="18"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
-      <c r="Z2" s="4"/>
-      <c r="AA2" s="4"/>
-      <c r="AB2" s="4"/>
-      <c r="AC2" s="4"/>
-      <c r="AD2" s="4"/>
-      <c r="AE2" s="4"/>
-      <c r="AF2" s="4"/>
-      <c r="AG2" s="4"/>
-      <c r="AH2" s="4"/>
-      <c r="AI2" s="4"/>
-      <c r="AJ2" s="4"/>
-      <c r="AK2" s="4"/>
-      <c r="AL2" s="4"/>
-      <c r="AM2" s="4"/>
-      <c r="AN2" s="4"/>
-      <c r="AO2" s="4"/>
+    <row r="2" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
     </row>
-    <row r="3" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="17" t="s">
+    <row r="3" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="18"/>
-      <c r="S3" s="18"/>
-      <c r="T3" s="18"/>
-      <c r="U3" s="18"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="4"/>
-      <c r="Z3" s="4"/>
-      <c r="AA3" s="4"/>
-      <c r="AB3" s="4"/>
-      <c r="AC3" s="4"/>
-      <c r="AD3" s="4"/>
-      <c r="AE3" s="4"/>
-      <c r="AF3" s="4"/>
-      <c r="AG3" s="4"/>
-      <c r="AH3" s="4"/>
-      <c r="AI3" s="4"/>
-      <c r="AJ3" s="4"/>
-      <c r="AK3" s="4"/>
-      <c r="AL3" s="4"/>
-      <c r="AM3" s="4"/>
-      <c r="AN3" s="4"/>
-      <c r="AO3" s="4"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12"/>
+      <c r="T3" s="12"/>
+      <c r="U3" s="12"/>
     </row>
-    <row r="4" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="19" t="s">
+    <row r="4" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="18"/>
-      <c r="P4" s="18"/>
-      <c r="Q4" s="18"/>
-      <c r="R4" s="18"/>
-      <c r="S4" s="18"/>
-      <c r="T4" s="18"/>
-      <c r="U4" s="18"/>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="4"/>
-      <c r="Y4" s="4"/>
-      <c r="Z4" s="4"/>
-      <c r="AA4" s="4"/>
-      <c r="AB4" s="4"/>
-      <c r="AC4" s="4"/>
-      <c r="AD4" s="4"/>
-      <c r="AE4" s="4"/>
-      <c r="AF4" s="4"/>
-      <c r="AG4" s="4"/>
-      <c r="AH4" s="4"/>
-      <c r="AI4" s="4"/>
-      <c r="AJ4" s="4"/>
-      <c r="AK4" s="4"/>
-      <c r="AL4" s="4"/>
-      <c r="AM4" s="4"/>
-      <c r="AN4" s="4"/>
-      <c r="AO4" s="4"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
     </row>
-    <row r="5" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="20" t="s">
+    <row r="5" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="21"/>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="21"/>
-      <c r="S5" s="21"/>
-      <c r="T5" s="21"/>
-      <c r="U5" s="21"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="4"/>
-      <c r="Y5" s="4"/>
-      <c r="Z5" s="4"/>
-      <c r="AA5" s="4"/>
-      <c r="AB5" s="4"/>
-      <c r="AC5" s="4"/>
-      <c r="AD5" s="4"/>
-      <c r="AE5" s="4"/>
-      <c r="AF5" s="4"/>
-      <c r="AG5" s="4"/>
-      <c r="AH5" s="4"/>
-      <c r="AI5" s="4"/>
-      <c r="AJ5" s="4"/>
-      <c r="AK5" s="4"/>
-      <c r="AL5" s="4"/>
-      <c r="AM5" s="4"/>
-      <c r="AN5" s="4"/>
-      <c r="AO5" s="4"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
+      <c r="S5" s="15"/>
+      <c r="T5" s="15"/>
+      <c r="U5" s="15"/>
     </row>
-    <row r="6" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="24" t="s">
+    <row r="6" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="24"/>
-      <c r="K6" s="24"/>
-      <c r="L6" s="24"/>
-      <c r="M6" s="24"/>
-      <c r="N6" s="24"/>
-      <c r="O6" s="22" t="s">
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
-      <c r="S6" s="18"/>
-      <c r="T6" s="18"/>
-      <c r="U6" s="18"/>
-      <c r="V6" s="4"/>
-      <c r="W6" s="4"/>
-      <c r="X6" s="4"/>
-      <c r="Y6" s="4"/>
-      <c r="Z6" s="4"/>
-      <c r="AA6" s="4"/>
-      <c r="AB6" s="4"/>
-      <c r="AC6" s="4"/>
-      <c r="AD6" s="4"/>
-      <c r="AE6" s="4"/>
-      <c r="AF6" s="4"/>
-      <c r="AG6" s="4"/>
-      <c r="AH6" s="4"/>
-      <c r="AI6" s="4"/>
-      <c r="AJ6" s="4"/>
-      <c r="AK6" s="4"/>
-      <c r="AL6" s="4"/>
-      <c r="AM6" s="4"/>
-      <c r="AN6" s="4"/>
-      <c r="AO6" s="4"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="12"/>
+      <c r="U6" s="12"/>
     </row>
-    <row r="7" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24" t="s">
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
-      <c r="K7" s="24"/>
-      <c r="L7" s="24"/>
-      <c r="M7" s="24"/>
-      <c r="N7" s="24"/>
-      <c r="O7" s="22" t="s">
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="22" t="s">
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="S7" s="18"/>
-      <c r="T7" s="18"/>
-      <c r="U7" s="18"/>
-      <c r="V7" s="4"/>
-      <c r="W7" s="4"/>
-      <c r="X7" s="4"/>
-      <c r="Y7" s="4"/>
-      <c r="Z7" s="4"/>
-      <c r="AA7" s="4"/>
-      <c r="AB7" s="4"/>
-      <c r="AC7" s="4"/>
-      <c r="AD7" s="4"/>
-      <c r="AE7" s="4"/>
-      <c r="AF7" s="4"/>
-      <c r="AG7" s="4"/>
-      <c r="AH7" s="4"/>
-      <c r="AI7" s="4"/>
-      <c r="AJ7" s="4"/>
-      <c r="AK7" s="4"/>
-      <c r="AL7" s="4"/>
-      <c r="AM7" s="4"/>
-      <c r="AN7" s="4"/>
-      <c r="AO7" s="4"/>
+      <c r="S7" s="12"/>
+      <c r="T7" s="12"/>
+      <c r="U7" s="12"/>
     </row>
-    <row r="8" spans="1:41" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="4" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -1089,7 +923,7 @@
       <c r="E8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="4" t="s">
         <v>22</v>
       </c>
       <c r="G8" s="1" t="s">
@@ -1101,7 +935,7 @@
       <c r="I8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K8" s="1" t="s">
@@ -1110,330 +944,191 @@
       <c r="L8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="M8" s="7" t="s">
+      <c r="M8" s="4" t="s">
         <v>22</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="O8" s="3" t="s">
+      <c r="O8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="P8" s="3" t="s">
+      <c r="P8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="Q8" s="3" t="s">
+      <c r="Q8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R8" s="3" t="s">
+      <c r="R8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="S8" s="3" t="s">
+      <c r="S8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="T8" s="3" t="s">
+      <c r="T8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="U8" s="3" t="s">
+      <c r="U8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="2"/>
-      <c r="Z8" s="2"/>
-      <c r="AA8" s="2"/>
-      <c r="AB8" s="2"/>
-      <c r="AC8" s="2"/>
-      <c r="AD8" s="2"/>
-      <c r="AE8" s="2"/>
-      <c r="AF8" s="2"/>
-      <c r="AG8" s="2"/>
-      <c r="AH8" s="2"/>
-      <c r="AI8" s="2"/>
-      <c r="AJ8" s="2"/>
-      <c r="AK8" s="2"/>
-      <c r="AL8" s="2"/>
-      <c r="AM8" s="2"/>
-      <c r="AN8" s="2"/>
-      <c r="AO8" s="2"/>
     </row>
-    <row r="9" spans="1:41" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="10" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="11"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="11"/>
-      <c r="R10" s="11"/>
-      <c r="S10" s="11"/>
-      <c r="T10" s="11"/>
-      <c r="U10" s="11"/>
-      <c r="V10" s="13"/>
-      <c r="W10" s="4"/>
-      <c r="X10" s="4" t="s">
+    <row r="9" spans="1:24" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="10" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
+      <c r="R10" s="7"/>
+      <c r="S10" s="7"/>
+      <c r="T10" s="7"/>
+      <c r="U10" s="7"/>
+      <c r="X10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Y10" s="4"/>
-      <c r="Z10" s="4"/>
-      <c r="AA10" s="4"/>
-      <c r="AB10" s="4"/>
-      <c r="AC10" s="4"/>
-      <c r="AD10" s="4"/>
-      <c r="AE10" s="4"/>
-      <c r="AF10" s="4"/>
-      <c r="AG10" s="4"/>
-      <c r="AH10" s="4"/>
-      <c r="AI10" s="4"/>
-      <c r="AJ10" s="4"/>
-      <c r="AK10" s="4"/>
-      <c r="AL10" s="4"/>
-      <c r="AM10" s="4"/>
-      <c r="AN10" s="4"/>
-      <c r="AO10" s="4"/>
     </row>
-    <row r="11" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="14"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="14"/>
-      <c r="O11" s="14"/>
-      <c r="P11" s="14"/>
-      <c r="Q11" s="14"/>
-      <c r="R11" s="14"/>
-      <c r="S11" s="14"/>
-      <c r="T11" s="14"/>
-      <c r="U11" s="14"/>
-      <c r="V11" s="16"/>
-      <c r="W11" s="4"/>
-      <c r="X11" s="4"/>
-      <c r="Y11" s="4"/>
-      <c r="Z11" s="4"/>
-      <c r="AA11" s="4"/>
-      <c r="AB11" s="4"/>
-      <c r="AC11" s="4"/>
-      <c r="AD11" s="4"/>
-      <c r="AE11" s="4"/>
-      <c r="AF11" s="4"/>
-      <c r="AG11" s="4"/>
-      <c r="AH11" s="4"/>
-      <c r="AI11" s="4"/>
-      <c r="AJ11" s="4"/>
-      <c r="AK11" s="4"/>
-      <c r="AL11" s="4"/>
-      <c r="AM11" s="4"/>
-      <c r="AN11" s="4"/>
-      <c r="AO11" s="4"/>
+    <row r="11" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
+      <c r="P11" s="9"/>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9"/>
+      <c r="S11" s="9"/>
+      <c r="T11" s="9"/>
+      <c r="U11" s="9"/>
     </row>
-    <row r="12" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="34"/>
-      <c r="B12" s="34"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="34"/>
-      <c r="N12" s="34"/>
-      <c r="O12" s="34"/>
-      <c r="P12" s="34"/>
-      <c r="Q12" s="34"/>
-      <c r="R12" s="34"/>
-      <c r="S12" s="34"/>
-      <c r="T12" s="34"/>
-      <c r="U12" s="34"/>
-      <c r="V12" s="6"/>
-      <c r="W12" s="6"/>
-      <c r="X12" s="6"/>
-      <c r="Y12" s="6"/>
-      <c r="Z12" s="6"/>
-      <c r="AA12" s="6"/>
-      <c r="AB12" s="6"/>
-      <c r="AC12" s="6"/>
-      <c r="AD12" s="6"/>
-      <c r="AE12" s="6"/>
-      <c r="AF12" s="6"/>
-      <c r="AG12" s="6"/>
-      <c r="AH12" s="6"/>
-      <c r="AI12" s="6"/>
-      <c r="AJ12" s="6"/>
-      <c r="AK12" s="6"/>
-      <c r="AL12" s="6"/>
-      <c r="AM12" s="6"/>
-      <c r="AN12" s="6"/>
-      <c r="AO12" s="6"/>
+    <row r="12" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="28"/>
+      <c r="L12" s="28"/>
+      <c r="M12" s="28"/>
+      <c r="N12" s="28"/>
+      <c r="O12" s="28"/>
+      <c r="P12" s="28"/>
+      <c r="Q12" s="28"/>
+      <c r="R12" s="28"/>
+      <c r="S12" s="28"/>
+      <c r="T12" s="28"/>
+      <c r="U12" s="28"/>
     </row>
-    <row r="13" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="35" t="s">
+    <row r="13" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="35"/>
-      <c r="L13" s="35"/>
-      <c r="M13" s="35"/>
-      <c r="N13" s="35"/>
-      <c r="O13" s="35"/>
-      <c r="P13" s="35"/>
-      <c r="Q13" s="35"/>
-      <c r="R13" s="35"/>
-      <c r="S13" s="35"/>
-      <c r="T13" s="35"/>
-      <c r="U13" s="35"/>
-      <c r="V13" s="6"/>
-      <c r="W13" s="6"/>
-      <c r="X13" s="6"/>
-      <c r="Y13" s="6"/>
-      <c r="Z13" s="6"/>
-      <c r="AA13" s="6"/>
-      <c r="AB13" s="6"/>
-      <c r="AC13" s="6"/>
-      <c r="AD13" s="6"/>
-      <c r="AE13" s="6"/>
-      <c r="AF13" s="6"/>
-      <c r="AG13" s="6"/>
-      <c r="AH13" s="6"/>
-      <c r="AI13" s="6"/>
-      <c r="AJ13" s="6"/>
-      <c r="AK13" s="6"/>
-      <c r="AL13" s="6"/>
-      <c r="AM13" s="6"/>
-      <c r="AN13" s="6"/>
-      <c r="AO13" s="6"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+      <c r="J13" s="29"/>
+      <c r="K13" s="29"/>
+      <c r="L13" s="29"/>
+      <c r="M13" s="29"/>
+      <c r="N13" s="29"/>
+      <c r="O13" s="29"/>
+      <c r="P13" s="29"/>
+      <c r="Q13" s="29"/>
+      <c r="R13" s="29"/>
+      <c r="S13" s="29"/>
+      <c r="T13" s="29"/>
+      <c r="U13" s="29"/>
     </row>
-    <row r="14" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
-      <c r="U14" s="10"/>
-      <c r="V14" s="6"/>
-      <c r="W14" s="6"/>
-      <c r="X14" s="6"/>
-      <c r="Y14" s="6"/>
-      <c r="Z14" s="6"/>
-      <c r="AA14" s="6"/>
-      <c r="AB14" s="6"/>
-      <c r="AC14" s="6"/>
-      <c r="AD14" s="6"/>
-      <c r="AE14" s="6"/>
-      <c r="AF14" s="6"/>
-      <c r="AG14" s="6"/>
-      <c r="AH14" s="6"/>
-      <c r="AI14" s="6"/>
-      <c r="AJ14" s="6"/>
-      <c r="AK14" s="6"/>
-      <c r="AL14" s="6"/>
-      <c r="AM14" s="6"/>
-      <c r="AN14" s="6"/>
-      <c r="AO14" s="6"/>
+    <row r="14" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6"/>
+      <c r="S14" s="6"/>
+      <c r="T14" s="6"/>
+      <c r="U14" s="6"/>
     </row>
-    <row r="15" spans="1:41" s="9" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="25" t="s">
+    <row r="15" spans="1:24" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="27" t="s">
+      <c r="B15" s="20"/>
+      <c r="C15" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="27" t="s">
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="J15" s="29"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
-      <c r="M15" s="30" t="s">
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
+      <c r="M15" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="N15" s="30"/>
-      <c r="O15" s="31"/>
-      <c r="P15" s="32" t="s">
+      <c r="N15" s="24"/>
+      <c r="O15" s="25"/>
+      <c r="P15" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="Q15" s="32"/>
-      <c r="R15" s="33" t="s">
+      <c r="Q15" s="26"/>
+      <c r="R15" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="S15" s="33"/>
-      <c r="T15" s="23" t="s">
+      <c r="S15" s="27"/>
+      <c r="T15" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="U15" s="23"/>
-      <c r="V15" s="8"/>
-      <c r="W15" s="8"/>
-      <c r="X15" s="8"/>
-      <c r="Y15" s="8"/>
-      <c r="Z15" s="8"/>
-      <c r="AA15" s="8"/>
-      <c r="AB15" s="8"/>
-      <c r="AC15" s="8"/>
-      <c r="AD15" s="8"/>
-      <c r="AE15" s="8"/>
-      <c r="AF15" s="8"/>
-      <c r="AG15" s="8"/>
-      <c r="AH15" s="8"/>
-      <c r="AI15" s="8"/>
-      <c r="AJ15" s="8"/>
-      <c r="AK15" s="8"/>
-      <c r="AL15" s="8"/>
-      <c r="AM15" s="8"/>
-      <c r="AN15" s="8"/>
-      <c r="AO15" s="8"/>
+      <c r="U15" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="19">

</xml_diff>

<commit_message>
Atualiza template v1 do relatório OSO
</commit_message>
<xml_diff>
--- a/tenants/sjc/reports/OSO/templates/v1.xlsx
+++ b/tenants/sjc/reports/OSO/templates/v1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaiqu\OneDrive\Área de Trabalho\Stravia Consultoria\01. Projetos\01.14 Goal Bus - API\Github\excel-report-api\tenants\sjc\reports\OSO\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CEAE44-B77D-4585-9C76-3AE93CAA3DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4826CD71-897F-449D-8FD4-2F330A11A969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3570" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="{{LINHA}}" sheetId="2" r:id="rId1"/>
@@ -125,9 +125,6 @@
     <t>{{LINHA}} - {{ITINERARIO}}</t>
   </si>
   <si>
-    <t>{{DESCRICAO_LINHA}}</t>
-  </si>
-  <si>
     <t>{{TIPO_DIA}}</t>
   </si>
   <si>
@@ -141,6 +138,9 @@
   </si>
   <si>
     <t>{{PONTO_FIM_COD}} - {{PONTO_FIM_DESCRICAO}}</t>
+  </si>
+  <si>
+    <t>{{TITULO_OSO}}</t>
   </si>
 </sst>
 </file>
@@ -388,22 +388,6 @@
     <xf numFmtId="20" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="20" fontId="8" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -431,11 +415,27 @@
     <xf numFmtId="20" fontId="8" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -727,185 +727,185 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="12"/>
-      <c r="S1" s="12"/>
-      <c r="T1" s="12"/>
-      <c r="U1" s="12"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
+      <c r="O1" s="23"/>
+      <c r="P1" s="23"/>
+      <c r="Q1" s="23"/>
+      <c r="R1" s="23"/>
+      <c r="S1" s="23"/>
+      <c r="T1" s="23"/>
+      <c r="U1" s="23"/>
     </row>
     <row r="2" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
     </row>
     <row r="3" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
+      <c r="A3" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23"/>
+      <c r="T3" s="23"/>
+      <c r="U3" s="23"/>
     </row>
     <row r="4" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
-      <c r="M4" s="12"/>
-      <c r="N4" s="12"/>
-      <c r="O4" s="12"/>
-      <c r="P4" s="12"/>
-      <c r="Q4" s="12"/>
-      <c r="R4" s="12"/>
-      <c r="S4" s="12"/>
-      <c r="T4" s="12"/>
-      <c r="U4" s="12"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="23"/>
+      <c r="T4" s="23"/>
+      <c r="U4" s="23"/>
     </row>
     <row r="5" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
-      <c r="S5" s="15"/>
-      <c r="T5" s="15"/>
-      <c r="U5" s="15"/>
+      <c r="A5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="29"/>
+      <c r="M5" s="29"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="29"/>
+      <c r="P5" s="29"/>
+      <c r="Q5" s="29"/>
+      <c r="R5" s="29"/>
+      <c r="S5" s="29"/>
+      <c r="T5" s="29"/>
+      <c r="U5" s="29"/>
     </row>
     <row r="6" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="16" t="s">
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="P6" s="12"/>
-      <c r="Q6" s="12"/>
-      <c r="R6" s="12"/>
-      <c r="S6" s="12"/>
-      <c r="T6" s="12"/>
-      <c r="U6" s="12"/>
+      <c r="P6" s="23"/>
+      <c r="Q6" s="23"/>
+      <c r="R6" s="23"/>
+      <c r="S6" s="23"/>
+      <c r="T6" s="23"/>
+      <c r="U6" s="23"/>
     </row>
     <row r="7" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
-      <c r="N7" s="18"/>
-      <c r="O7" s="16" t="s">
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="P7" s="12"/>
-      <c r="Q7" s="12"/>
-      <c r="R7" s="16" t="s">
+      <c r="P7" s="23"/>
+      <c r="Q7" s="23"/>
+      <c r="R7" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="S7" s="12"/>
-      <c r="T7" s="12"/>
-      <c r="U7" s="12"/>
+      <c r="S7" s="23"/>
+      <c r="T7" s="23"/>
+      <c r="U7" s="23"/>
     </row>
     <row r="8" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -1023,52 +1023,52 @@
       <c r="U11" s="9"/>
     </row>
     <row r="12" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="28"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
-      <c r="K12" s="28"/>
-      <c r="L12" s="28"/>
-      <c r="M12" s="28"/>
-      <c r="N12" s="28"/>
-      <c r="O12" s="28"/>
-      <c r="P12" s="28"/>
-      <c r="Q12" s="28"/>
-      <c r="R12" s="28"/>
-      <c r="S12" s="28"/>
-      <c r="T12" s="28"/>
-      <c r="U12" s="28"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
+      <c r="L12" s="24"/>
+      <c r="M12" s="24"/>
+      <c r="N12" s="24"/>
+      <c r="O12" s="24"/>
+      <c r="P12" s="24"/>
+      <c r="Q12" s="24"/>
+      <c r="R12" s="24"/>
+      <c r="S12" s="24"/>
+      <c r="T12" s="24"/>
+      <c r="U12" s="24"/>
     </row>
     <row r="13" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
-      <c r="J13" s="29"/>
-      <c r="K13" s="29"/>
-      <c r="L13" s="29"/>
-      <c r="M13" s="29"/>
-      <c r="N13" s="29"/>
-      <c r="O13" s="29"/>
-      <c r="P13" s="29"/>
-      <c r="Q13" s="29"/>
-      <c r="R13" s="29"/>
-      <c r="S13" s="29"/>
-      <c r="T13" s="29"/>
-      <c r="U13" s="29"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="25"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="25"/>
+      <c r="M13" s="25"/>
+      <c r="N13" s="25"/>
+      <c r="O13" s="25"/>
+      <c r="P13" s="25"/>
+      <c r="Q13" s="25"/>
+      <c r="R13" s="25"/>
+      <c r="S13" s="25"/>
+      <c r="T13" s="25"/>
+      <c r="U13" s="25"/>
     </row>
     <row r="14" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6"/>
@@ -1094,44 +1094,49 @@
       <c r="U14" s="6"/>
     </row>
     <row r="15" spans="1:24" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="21" t="s">
+      <c r="B15" s="14"/>
+      <c r="C15" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="24" t="s">
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="N15" s="24"/>
-      <c r="O15" s="25"/>
-      <c r="P15" s="26" t="s">
+      <c r="N15" s="18"/>
+      <c r="O15" s="19"/>
+      <c r="P15" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="Q15" s="26"/>
-      <c r="R15" s="27" t="s">
+      <c r="Q15" s="20"/>
+      <c r="R15" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="S15" s="27"/>
-      <c r="T15" s="17" t="s">
+      <c r="S15" s="21"/>
+      <c r="T15" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="U15" s="17"/>
+      <c r="U15" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A1:U2"/>
+    <mergeCell ref="A3:U3"/>
+    <mergeCell ref="A4:U4"/>
+    <mergeCell ref="A5:U5"/>
+    <mergeCell ref="O6:U6"/>
     <mergeCell ref="T15:U15"/>
     <mergeCell ref="A6:N6"/>
     <mergeCell ref="A7:G7"/>
@@ -1146,11 +1151,6 @@
     <mergeCell ref="R7:U7"/>
     <mergeCell ref="A12:U12"/>
     <mergeCell ref="A13:U13"/>
-    <mergeCell ref="A1:U2"/>
-    <mergeCell ref="A3:U3"/>
-    <mergeCell ref="A4:U4"/>
-    <mergeCell ref="A5:U5"/>
-    <mergeCell ref="O6:U6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
@@ -1160,14 +1160,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b68611d9-97ec-4b72-b536-39046913c13e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="5b2e1221-979e-4305-8561-548309efb779" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1432,21 +1430,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b68611d9-97ec-4b72-b536-39046913c13e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="5b2e1221-979e-4305-8561-548309efb779" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89BAA058-C7F0-45A3-9958-90E90184B301}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28D29668-C75A-4B4D-96BA-75B2C8869B64}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b68611d9-97ec-4b72-b536-39046913c13e"/>
-    <ds:schemaRef ds:uri="5b2e1221-979e-4305-8561-548309efb779"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1471,9 +1468,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28D29668-C75A-4B4D-96BA-75B2C8869B64}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89BAA058-C7F0-45A3-9958-90E90184B301}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b68611d9-97ec-4b72-b536-39046913c13e"/>
+    <ds:schemaRef ds:uri="5b2e1221-979e-4305-8561-548309efb779"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>